<commit_message>
Add versioning for requirement
</commit_message>
<xml_diff>
--- a/resource/groundTruths/decision/CF_M08_ground_truth_decision.xlsx
+++ b/resource/groundTruths/decision/CF_M08_ground_truth_decision.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oguzarslan/Desktop/upc/semester-4/Thesis/MappingGenerator/resource/groundTruths/decision/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38E3A6EF-BA24-A94E-901C-E3A2438A5C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A6BE0CDA-FC3C-DF4C-B543-48135B8B32E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10780" yWindow="940" windowWidth="18620" windowHeight="16420" xr2:uid="{62E08A4D-93B2-534F-834C-F4E19BDCC923}"/>
   </bookViews>
@@ -149,9 +149,6 @@
     <t>*CF_M08_C10</t>
   </si>
   <si>
-    <t>*CF_M08_C11, *CF_M08_C12</t>
-  </si>
-  <si>
     <t>*CF_M08_C14</t>
   </si>
   <si>
@@ -204,6 +201,9 @@
   </si>
   <si>
     <t>*CF_M08_C21, CF_M08_C05</t>
+  </si>
+  <si>
+    <t>*CF_M08_C11, *CF_M08_C12, *CF_M08_C13</t>
   </si>
 </sst>
 </file>
@@ -682,7 +682,7 @@
         <v>15</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="E2" s="7" t="s">
         <v>7</v>
@@ -722,7 +722,7 @@
         <v>16</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>37</v>
+        <v>55</v>
       </c>
       <c r="E4" s="7" t="s">
         <v>8</v>
@@ -742,7 +742,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E5" s="7" t="s">
         <v>9</v>
@@ -762,7 +762,7 @@
         <v>17</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="E6" s="7" t="s">
         <v>10</v>
@@ -782,7 +782,7 @@
         <v>17</v>
       </c>
       <c r="D7" s="9" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>11</v>
@@ -802,7 +802,7 @@
         <v>17</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E8" s="7" t="s">
         <v>20</v>
@@ -822,7 +822,7 @@
         <v>18</v>
       </c>
       <c r="D9" s="9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E9" s="7" t="s">
         <v>12</v>
@@ -842,7 +842,7 @@
         <v>18</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E10" s="7" t="s">
         <v>13</v>
@@ -862,7 +862,7 @@
         <v>19</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E11" s="7" t="s">
         <v>14</v>
@@ -882,7 +882,7 @@
         <v>19</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E12" s="7" t="s">
         <v>21</v>
@@ -902,7 +902,7 @@
         <v>19</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E13" s="7" t="s">
         <v>22</v>
@@ -916,16 +916,16 @@
         <v>6</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F14" s="9">
         <v>67</v>
@@ -936,16 +936,16 @@
         <v>6</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C15" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="E15" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="D15" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>54</v>
       </c>
       <c r="F15" s="9">
         <v>66</v>

</xml_diff>